<commit_message>
everything up to date working as far as I can tell, added more baud filtering to correct any errors in reading authority from CTC as there is some randomness just based on the CTC is only able to tell what block the train is on and nothing else
</commit_message>
<xml_diff>
--- a/full_integration/assets/Train_Scheduling.xlsx
+++ b/full_integration/assets/Train_Scheduling.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samar\OneDrive\Desktop\University of Pittsburgh\Year 4\SystemsAndProjectEng\Systems-Engineering-ECE1140\full_integration\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/lao57_pitt_edu/Documents/CODE_folder/1140 code/Systems-Engineering-ECE1140/Track_Model_controller_integration/Systems-Engineering-ECE1140/full_integration/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F2FF7E-C2C4-4400-9614-8870773A8AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{98F2FF7E-C2C4-4400-9614-8870773A8AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{980B37B4-2031-4D79-9C6F-E7D1DC9FF4E4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Red Line Scheduling" sheetId="1" r:id="rId1"/>
@@ -32,10 +32,10 @@
     <t>expected_arrival_times</t>
   </si>
   <si>
-    <t>7:30, 7:45</t>
+    <t>7:30, 7:45, 8:00</t>
   </si>
   <si>
-    <t>EDGEBROOK, YARD</t>
+    <t>DORMONT,GLENBURY, YARD</t>
   </si>
 </sst>
 </file>
@@ -122,6 +122,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,12 +417,12 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="3" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="13.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -440,14 +444,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.52734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.52734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.52734375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -458,7 +462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="3">
         <v>101</v>
       </c>

</xml_diff>

<commit_message>
added mid block correction to baud pickpup to avoid errors from stations on smaller blocks fixes the error on central
</commit_message>
<xml_diff>
--- a/full_integration/assets/Train_Scheduling.xlsx
+++ b/full_integration/assets/Train_Scheduling.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samar\OneDrive\Desktop\University of Pittsburgh\Year 4\SystemsAndProjectEng\Systems-Engineering-ECE1140\full_integration\assets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD03ECD-4974-4435-B086-1EA083627561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Red Line Scheduling"/>
-    <sheet r:id="rId2" sheetId="2" name="Green Line Scheduling"/>
+    <sheet name="Red Line Scheduling" sheetId="1" r:id="rId1"/>
+    <sheet name="Green Line Scheduling" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Train ID</t>
   </si>
@@ -35,14 +41,49 @@
     <t>DORMONT,GLENBURY, YARD</t>
   </si>
   <si>
-    <t>7:30, 8:00, 8:30</t>
+    <t>8:30, 9:00, 9:30</t>
+  </si>
+  <si>
+    <t>9:00, 9:30, 10:00</t>
+  </si>
+  <si>
+    <t>DORMONT, EDGEBROOK, YARD</t>
+  </si>
+  <si>
+    <t>9:30, 10:00</t>
+  </si>
+  <si>
+    <t>DORMONT, YARD</t>
+  </si>
+  <si>
+    <t>GLENBURY, CENTRAL, YARD</t>
+  </si>
+  <si>
+    <t>DORMONT, PIONEER, YARD</t>
+  </si>
+  <si>
+    <t>7:30, 8:30</t>
+  </si>
+  <si>
+    <t>11:00, 11:30, 12:00</t>
+  </si>
+  <si>
+    <t>12:30, 13:00, 13:30</t>
+  </si>
+  <si>
+    <t>13:00, 13:30, 14:00</t>
+  </si>
+  <si>
+    <t>13:30, 14:00</t>
+  </si>
+  <si>
+    <t>10:00, 10:30, 11:30</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -91,44 +132,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -139,10 +171,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -180,71 +212,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -272,7 +304,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -295,11 +327,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -308,13 +340,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -324,7 +356,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -333,7 +365,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -342,7 +374,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -350,10 +382,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -418,26 +450,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="3" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -447,49 +477,137 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="31.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.54296875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="4">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
+        <v>1001</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>901</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
+        <v>801</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>701</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>601</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>501</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>401</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>301</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
         <v>201</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="1">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1">
         <v>101</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>6</v>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>